<commit_message>
Fix Origin Dialga/Palkia to GO-only shiny
Their Origin Forme needs the Adamant Crystal / Lustrous Globe, which exist only
in Legends: Arceus where Dialga/Palkia are shiny-locked — so (unlike Giratina,
whose Griseous Orb is in BDSP alongside a huntable shiny) a shiny Origin
Dialga/Palkia can't be self-caught. Dropped their spurious Home OT channel;
they now correctly offer only GO. Verified in-browser: base Dialga/Palkia stay
OT+GO, Origin formes show GO only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mtz18idK3joeBU4SzZCbtU
</commit_message>
<xml_diff>
--- a/data/pokemon-shiny/legendary_mythical_shiny_master.xlsx
+++ b/data/pokemon-shiny/legendary_mythical_shiny_master.xlsx
@@ -14920,7 +14920,7 @@
       </c>
       <c r="Y114" t="inlineStr">
         <is>
-          <t>Separate shiny raid boss in GO; main-series Origin form via the Adamant Crystal.</t>
+          <t>GO-ONLY shiny. Unlike Giratina, a shiny Origin Dialga can only come from Pokémon GO: the Adamant Crystal is PLA-exclusive and the PLA Dialga is shiny-locked, so it can't be paired with a huntable shiny.</t>
         </is>
       </c>
     </row>
@@ -15047,7 +15047,7 @@
       </c>
       <c r="Y115" t="inlineStr">
         <is>
-          <t>Separate shiny raid boss in GO; main-series Origin form via the Lustrous Globe.</t>
+          <t>GO-ONLY shiny. Unlike Giratina, a shiny Origin Palkia can only come from Pokémon GO: the Lustrous Globe is PLA-exclusive and the PLA Palkia is shiny-locked, so it can't be paired with a huntable shiny.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Type: Null, Silvally, Poipole, Naganadel — they ARE huntable
The Gen 7 GIFT versions aren't shiny-locked (verified across GameFAQs, PokémonDB,
Project Pokemon, FBTB):
- Type: Null — Gladion's gift in Sun/Moon & USUM is soft-reset huntable at full
  odds (only the SwSh gift is locked).
- Poipole — the USUM Ultra Recon Squad gift is soft-reset huntable (SwSh Crown
  Tundra and GO versions are locked).
- Silvally / Naganadel — huntable by evolving the hunted shiny pre-evo; Silvally
  also had a 2017 event distribution.
Cosmog/Cosmoem verified to STAY shiny-locked (Nebby is locked in SM/USUM), so
they remain unavailable.

Counts: shiny exists 69->70, never 25->24, RNG-huntable ever 61->63, currently
huntable 56->58; all 11 Ultra Beasts now huntable.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mtz18idK3joeBU4SzZCbtU
</commit_message>
<xml_diff>
--- a/data/pokemon-shiny/legendary_mythical_shiny_master.xlsx
+++ b/data/pokemon-shiny/legendary_mythical_shiny_master.xlsx
@@ -7454,22 +7454,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>D (shiny unavailable)</t>
+          <t>A (true hunt, current)</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>shiny-locked</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sun:1/4096</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>Officially 'Synthetic Pokémon'; Bulbapedia counts it as Legendary. No legit shiny Type: Null: the gift is shiny-locked everywhere, and the 2017 event distributed the already-evolved Shiny SILVALLY (you cannot devolve it). So shiny Silvally exists, but shiny Type: Null does not.</t>
+          <t>Correction: shiny Type: Null IS huntable — Gladion's gift in Sun/Moon &amp; Ultra Sun/Ultra Moon is not shiny-locked (soft-reset, full odds; gifts ignore the Shiny Charm). Only the SwSh gift is locked.</t>
         </is>
       </c>
     </row>
@@ -7586,22 +7586,22 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>C (event distribution only)</t>
+          <t>A (true hunt, current)</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sun:1/4096</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="Y57" t="inlineStr">
         <is>
-          <t>Correction: a legit shiny Silvally EXISTS via the official 2017 GameStop/GAME/EB event distribution (already evolved) — but it is NOT RNG-huntable. The in-game Type: Null gift is shiny-locked everywhere.</t>
+          <t>Correction: shiny Silvally IS huntable — evolve a soft-reset shiny Type: Null from Sun/Moon or USUM (the Gen 7 gift isn't locked). A guaranteed shiny was also officially distributed in 2017.</t>
         </is>
       </c>
     </row>
@@ -13677,22 +13677,22 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>D (shiny unavailable)</t>
+          <t>A (true hunt, current)</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -13732,7 +13732,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>shiny-locked</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -13747,7 +13747,7 @@
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ultra Sun:1/4096</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -13777,7 +13777,7 @@
       </c>
       <c r="Y105" t="inlineStr">
         <is>
-          <t>Ultra Beast. Shiny UNAVAILABLE (shiny-locked in both USUM and GO).</t>
+          <t>Correction: shiny Poipole IS huntable — the Ultra Sun/Ultra Moon Ultra Recon Squad gift is not shiny-locked (soft-reset, full odds). Shiny-locked in SwSh Crown Tundra and in GO.</t>
         </is>
       </c>
     </row>
@@ -13804,22 +13804,22 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>D (shiny unavailable)</t>
+          <t>A (true hunt, current)</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -13874,7 +13874,7 @@
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ultra Sun:1/4096</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V106" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="Y106" t="inlineStr">
         <is>
-          <t>Ultra Beast. Shiny UNAVAILABLE (only from shiny-locked Poipole).</t>
+          <t>Correction: shiny Naganadel IS huntable — evolve a soft-reset shiny Poipole from USUM. Shiny-locked in GO.</t>
         </is>
       </c>
     </row>

</xml_diff>